<commit_message>
Fix Google Sheets date validation formula error by using native date cell formatting
</commit_message>
<xml_diff>
--- a/LAXMTB_Race_Data.xlsx
+++ b/LAXMTB_Race_Data.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="90">
   <si>
     <t>--- SCHEDULE ---</t>
   </si>
@@ -47,9 +47,6 @@
     <t>Friday</t>
   </si>
   <si>
-    <t>2026-09-04</t>
-  </si>
-  <si>
     <t>3:00 PM</t>
   </si>
   <si>
@@ -65,9 +62,6 @@
     <t>Saturday</t>
   </si>
   <si>
-    <t>2026-09-05</t>
-  </si>
-  <si>
     <t>8:00 AM</t>
   </si>
   <si>
@@ -122,9 +116,6 @@
     <t>Sunday</t>
   </si>
   <si>
-    <t>2026-09-06</t>
-  </si>
-  <si>
     <t>7:00 AM</t>
   </si>
   <si>
@@ -155,9 +146,6 @@
     <t>Monday</t>
   </si>
   <si>
-    <t>2026-09-07</t>
-  </si>
-  <si>
     <t>Morning</t>
   </si>
   <si>
@@ -215,21 +203,12 @@
     <t>Leashed Pets Only: Dogs prohibited in active course areas and staging grid zones.</t>
   </si>
   <si>
-    <t>2026-09-11</t>
-  </si>
-  <si>
     <t>1:00 PM</t>
   </si>
   <si>
     <t>Pit Zone Setup, Pre-Ride &amp; CAMBA Trail Tour</t>
   </si>
   <si>
-    <t>2026-09-12</t>
-  </si>
-  <si>
-    <t>2026-09-13</t>
-  </si>
-  <si>
     <t>9:00 AM</t>
   </si>
   <si>
@@ -251,24 +230,15 @@
     <t>Village Camping: Mt. Telemark festival camping available on-site (advance booking recommended).</t>
   </si>
   <si>
-    <t>2026-09-25</t>
-  </si>
-  <si>
     <t>2:00 PM</t>
   </si>
   <si>
     <t>Pre-Ride Open &amp; Pit Zone Setup</t>
   </si>
   <si>
-    <t>2026-09-26</t>
-  </si>
-  <si>
     <t>South Conference Racing</t>
   </si>
   <si>
-    <t>2026-09-27</t>
-  </si>
-  <si>
     <t>Pre-Ride Open</t>
   </si>
   <si>
@@ -284,15 +254,6 @@
     <t>Spectators: Excellent viewing points along West and East Singletrack loops.</t>
   </si>
   <si>
-    <t>2026-10-02</t>
-  </si>
-  <si>
-    <t>2026-10-03</t>
-  </si>
-  <si>
-    <t>2026-10-04</t>
-  </si>
-  <si>
     <t>Course Pre-Ride</t>
   </si>
   <si>
@@ -305,22 +266,13 @@
     <t>Parking: Park only in designated grassy farm pastures as directed by volunteers.</t>
   </si>
   <si>
-    <t>2026-10-16</t>
-  </si>
-  <si>
     <t>12:00 PM</t>
   </si>
   <si>
     <t>State Championship Pre-Ride &amp; Night Ride Festivities</t>
   </si>
   <si>
-    <t>2026-10-17</t>
-  </si>
-  <si>
     <t>High School State Championship Finals &amp; Night Pump Track</t>
-  </si>
-  <si>
-    <t>2026-10-18</t>
   </si>
   <si>
     <t>8:30 AM</t>
@@ -344,7 +296,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="h:mm AM/PM"/>
+    <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -411,13 +363,13 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -429,7 +381,7 @@
       <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="h:mm AM/PM"/>
+      <numFmt numFmtId="165" formatCode="@"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -909,13 +861,15 @@
   <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="4" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" style="1" customWidth="1"/>
+    <col min="3" max="4" width="14.7109375" style="2" customWidth="1"/>
     <col min="5" max="5" width="48.7109375" customWidth="1"/>
     <col min="6" max="7" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
@@ -923,13 +877,13 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E2" t="s">
@@ -946,330 +900,326 @@
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1">
+        <v>46269</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="2"/>
+      <c r="E3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="3"/>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>11</v>
       </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="1">
+        <v>46270</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="E4" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="F4" t="s">
         <v>17</v>
       </c>
-      <c r="E4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" t="s">
-        <v>19</v>
-      </c>
       <c r="G4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="1">
+        <v>46270</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="E5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" t="s">
-        <v>22</v>
-      </c>
       <c r="G5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1">
+        <v>46270</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="F6" t="s">
         <v>24</v>
       </c>
-      <c r="E6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" t="s">
-        <v>26</v>
-      </c>
       <c r="G6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="1">
+        <v>46270</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="3"/>
-      <c r="E7" t="s">
+      <c r="G7" t="s">
         <v>28</v>
-      </c>
-      <c r="F7" t="s">
-        <v>29</v>
-      </c>
-      <c r="G7" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="1">
+        <v>46270</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="E8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F8" t="s">
-        <v>26</v>
-      </c>
       <c r="G8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="1">
+        <v>46271</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" t="s">
-        <v>36</v>
-      </c>
       <c r="F9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="1">
+        <v>46271</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="E10" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E10" t="s">
-        <v>38</v>
-      </c>
       <c r="F10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D11" s="3"/>
+        <v>31</v>
+      </c>
+      <c r="B11" s="1">
+        <v>46271</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="2"/>
       <c r="E11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" s="3"/>
+        <v>31</v>
+      </c>
+      <c r="B12" s="1">
+        <v>46271</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="2"/>
       <c r="E12" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F12" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="G12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="1">
+        <v>46272</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" s="2"/>
+      <c r="E13" t="s">
+        <v>43</v>
+      </c>
+      <c r="F13" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="3" t="s">
         <v>44</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D13" s="3"/>
-      <c r="E13" t="s">
-        <v>47</v>
-      </c>
-      <c r="F13" t="s">
-        <v>12</v>
-      </c>
-      <c r="G13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>49</v>
-      </c>
-      <c r="B17" t="s">
-        <v>50</v>
+        <v>45</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24" s="1" t="s">
-        <v>58</v>
+      <c r="A24" s="3" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
+  <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A3:A50">
       <formula1>"Friday,Saturday,Sunday,Monday"</formula1>
-    </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B50">
-      <formula1>2026-01-01</formula1>
-      <formula2>2026-12-31</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F3:F50">
       <formula1>"Pre-Ride,Racing,Team Event,Spectating,Team Ride,Venue,Awards,Meeting,Other"</formula1>
@@ -1301,13 +1251,15 @@
   <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="4" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" style="1" customWidth="1"/>
+    <col min="3" max="4" width="14.7109375" style="2" customWidth="1"/>
     <col min="5" max="5" width="48.7109375" customWidth="1"/>
     <col min="6" max="7" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1315,13 +1267,13 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E2" t="s">
@@ -1338,223 +1290,219 @@
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>24</v>
+      <c r="B3" s="1">
+        <v>46276</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="F3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="1">
+        <v>46277</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="F4" t="s">
         <v>17</v>
       </c>
-      <c r="E4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" t="s">
-        <v>19</v>
-      </c>
       <c r="G4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="1">
+        <v>46277</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="E5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
         <v>28</v>
-      </c>
-      <c r="F5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="1">
+        <v>46278</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" t="s">
-        <v>36</v>
-      </c>
       <c r="F6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>70</v>
+        <v>31</v>
+      </c>
+      <c r="B7" s="1">
+        <v>46278</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>63</v>
       </c>
       <c r="E7" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="F7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="3"/>
+        <v>31</v>
+      </c>
+      <c r="B8" s="1">
+        <v>46278</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="2"/>
       <c r="E8" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F8" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D9" s="3"/>
+        <v>31</v>
+      </c>
+      <c r="B9" s="1">
+        <v>46278</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="2"/>
       <c r="E9" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="F9" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="G9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="1" t="s">
-        <v>48</v>
+      <c r="A12" s="3" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>49</v>
-      </c>
-      <c r="B13" t="s">
-        <v>50</v>
+        <v>45</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:1">
-      <c r="A20" s="1" t="s">
-        <v>58</v>
+      <c r="A20" s="3" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24" spans="1:1">
       <c r="A24" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
+  <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A3:A50">
       <formula1>"Friday,Saturday,Sunday,Monday"</formula1>
-    </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B50">
-      <formula1>2026-01-01</formula1>
-      <formula2>2026-12-31</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F3:F50">
       <formula1>"Pre-Ride,Racing,Team Event,Spectating,Team Ride,Venue,Awards,Meeting,Other"</formula1>
@@ -1581,13 +1529,15 @@
   <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="4" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" style="1" customWidth="1"/>
+    <col min="3" max="4" width="14.7109375" style="2" customWidth="1"/>
     <col min="5" max="5" width="48.7109375" customWidth="1"/>
     <col min="6" max="7" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1595,13 +1545,13 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E2" t="s">
@@ -1618,223 +1568,219 @@
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>24</v>
+      <c r="B3" s="1">
+        <v>46290</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="F3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="1">
+        <v>46291</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" t="s">
+        <v>72</v>
+      </c>
+      <c r="F4" t="s">
         <v>17</v>
       </c>
-      <c r="E4" t="s">
-        <v>81</v>
-      </c>
-      <c r="F4" t="s">
-        <v>19</v>
-      </c>
       <c r="G4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="1">
+        <v>46291</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="E5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
         <v>28</v>
-      </c>
-      <c r="F5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="1">
+        <v>46292</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" t="s">
-        <v>36</v>
-      </c>
       <c r="F6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>70</v>
+        <v>31</v>
+      </c>
+      <c r="B7" s="1">
+        <v>46292</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>63</v>
       </c>
       <c r="E7" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="F7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="3"/>
+        <v>31</v>
+      </c>
+      <c r="B8" s="1">
+        <v>46292</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="2"/>
       <c r="E8" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F8" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D9" s="3"/>
+        <v>31</v>
+      </c>
+      <c r="B9" s="1">
+        <v>46292</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="2"/>
       <c r="E9" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="F9" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="G9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="1" t="s">
-        <v>48</v>
+      <c r="A12" s="3" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>49</v>
-      </c>
-      <c r="B13" t="s">
-        <v>50</v>
+        <v>45</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:1">
-      <c r="A20" s="1" t="s">
-        <v>58</v>
+      <c r="A20" s="3" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
     </row>
     <row r="24" spans="1:1">
       <c r="A24" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
+  <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A3:A50">
       <formula1>"Friday,Saturday,Sunday,Monday"</formula1>
-    </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B50">
-      <formula1>2026-01-01</formula1>
-      <formula2>2026-12-31</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F3:F50">
       <formula1>"Pre-Ride,Racing,Team Event,Spectating,Team Ride,Venue,Awards,Meeting,Other"</formula1>
@@ -1861,13 +1807,15 @@
   <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="4" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" style="1" customWidth="1"/>
+    <col min="3" max="4" width="14.7109375" style="2" customWidth="1"/>
     <col min="5" max="5" width="48.7109375" customWidth="1"/>
     <col min="6" max="7" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1875,13 +1823,13 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E2" t="s">
@@ -1898,223 +1846,219 @@
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>24</v>
+      <c r="B3" s="1">
+        <v>46297</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="F3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="1">
+        <v>46298</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" t="s">
+        <v>72</v>
+      </c>
+      <c r="F4" t="s">
         <v>17</v>
       </c>
-      <c r="E4" t="s">
-        <v>81</v>
-      </c>
-      <c r="F4" t="s">
-        <v>19</v>
-      </c>
       <c r="G4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="1">
+        <v>46298</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="E5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
         <v>28</v>
-      </c>
-      <c r="F5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="1">
+        <v>46299</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" t="s">
-        <v>36</v>
-      </c>
       <c r="F6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>70</v>
+        <v>31</v>
+      </c>
+      <c r="B7" s="1">
+        <v>46299</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>63</v>
       </c>
       <c r="E7" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="F7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="3"/>
+        <v>31</v>
+      </c>
+      <c r="B8" s="1">
+        <v>46299</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="2"/>
       <c r="E8" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F8" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D9" s="3"/>
+        <v>31</v>
+      </c>
+      <c r="B9" s="1">
+        <v>46299</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="2"/>
       <c r="E9" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="F9" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="G9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="1" t="s">
-        <v>48</v>
+      <c r="A12" s="3" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>49</v>
-      </c>
-      <c r="B13" t="s">
-        <v>50</v>
+        <v>45</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:1">
-      <c r="A20" s="1" t="s">
-        <v>58</v>
+      <c r="A20" s="3" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24" spans="1:1">
       <c r="A24" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
+  <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A3:A50">
       <formula1>"Friday,Saturday,Sunday,Monday"</formula1>
-    </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B50">
-      <formula1>2026-01-01</formula1>
-      <formula2>2026-12-31</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F3:F50">
       <formula1>"Pre-Ride,Racing,Team Event,Spectating,Team Ride,Venue,Awards,Meeting,Other"</formula1>
@@ -2141,13 +2085,15 @@
   <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="4" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" style="1" customWidth="1"/>
+    <col min="3" max="4" width="14.7109375" style="2" customWidth="1"/>
     <col min="5" max="5" width="48.7109375" customWidth="1"/>
     <col min="6" max="7" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
@@ -2155,13 +2101,13 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E2" t="s">
@@ -2178,179 +2124,175 @@
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>27</v>
+      <c r="B3" s="1">
+        <v>46311</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="F3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="1">
+        <v>46312</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>17</v>
+      <c r="D4" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="E4" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="F4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="C5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="1">
+        <v>46312</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="E5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
         <v>28</v>
-      </c>
-      <c r="F5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="1">
+        <v>46313</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" t="s">
-        <v>36</v>
-      </c>
       <c r="F6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="D7" s="3"/>
+        <v>31</v>
+      </c>
+      <c r="B7" s="1">
+        <v>46313</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D7" s="2"/>
       <c r="E7" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="F7" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:7">
-      <c r="A10" s="1" t="s">
-        <v>48</v>
+      <c r="A10" s="3" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>49</v>
-      </c>
-      <c r="B11" t="s">
-        <v>50</v>
+        <v>45</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="1:1">
-      <c r="A18" s="1" t="s">
-        <v>58</v>
+      <c r="A18" s="3" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
+  <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A3:A50">
       <formula1>"Friday,Saturday,Sunday,Monday"</formula1>
-    </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B50">
-      <formula1>2026-01-01</formula1>
-      <formula2>2026-12-31</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F3:F50">
       <formula1>"Pre-Ride,Racing,Team Event,Spectating,Team Ride,Venue,Awards,Meeting,Other"</formula1>

</xml_diff>